<commit_message>
Add biodiversity pricing support and paper4 assets
</commit_message>
<xml_diff>
--- a/myCode/Ag2050/2_processed_data/labour_cost_forecast.xlsx
+++ b/myCode/Ag2050/2_processed_data/labour_cost_forecast.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,6 +454,36 @@
           <t>Very_High</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Historical</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Fitted</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Plot_Low</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Plot_Medium</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Plot_High</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Plot_Very_High</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -471,6 +501,24 @@
       <c r="E2" t="n">
         <v>1</v>
       </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.9369887862582014</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -488,6 +536,24 @@
       <c r="E3" t="n">
         <v>1</v>
       </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.9769583215142472</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -505,6 +571,24 @@
       <c r="E4" t="n">
         <v>1</v>
       </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.016124595359883</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -522,6 +606,24 @@
       <c r="E5" t="n">
         <v>1</v>
       </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1.054503673026557</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -539,6 +641,24 @@
       <c r="E6" t="n">
         <v>1</v>
       </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1.092111298448804</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -556,6 +676,24 @@
       <c r="E7" t="n">
         <v>1.153908543682574</v>
       </c>
+      <c r="F7" t="n">
+        <v>1.153908543682574</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.128962900690027</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -573,6 +711,24 @@
       <c r="E8" t="n">
         <v>1.14257096572451</v>
       </c>
+      <c r="F8" t="n">
+        <v>1.14257096572451</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.165088992602441</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -590,6 +746,24 @@
       <c r="E9" t="n">
         <v>1.208048138561229</v>
       </c>
+      <c r="F9" t="n">
+        <v>1.208048138561229</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1.200487865980228</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -607,6 +781,24 @@
       <c r="E10" t="n">
         <v>1.215777713114327</v>
       </c>
+      <c r="F10" t="n">
+        <v>1.215777713114327</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1.235181724758443</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -624,6 +816,24 @@
       <c r="E11" t="n">
         <v>1.358509372339871</v>
       </c>
+      <c r="F11" t="n">
+        <v>1.358509372339871</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.269179024863056</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -641,6 +851,24 @@
       <c r="E12" t="n">
         <v>1.105484425759602</v>
       </c>
+      <c r="F12" t="n">
+        <v>1.105484425759602</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1.302507214468904</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -658,6 +886,24 @@
       <c r="E13" t="n">
         <v>1.276148524225631</v>
       </c>
+      <c r="F13" t="n">
+        <v>1.276148524225631</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1.335140381698887</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -675,6 +921,24 @@
       <c r="E14" t="n">
         <v>1.49238768827198</v>
       </c>
+      <c r="F14" t="n">
+        <v>1.49238768827198</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1.367134294053697</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -692,6 +956,24 @@
       <c r="E15" t="n">
         <v>1.438405529593662</v>
       </c>
+      <c r="F15" t="n">
+        <v>1.438405529593662</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1.398506635930348</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -709,22 +991,58 @@
       <c r="E16" t="n">
         <v>1.471446502093358</v>
       </c>
+      <c r="F16" t="n">
+        <v>1.471446502093358</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1.429243246417209</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1.341575415210259</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1.429243246417209</v>
+      </c>
+      <c r="J16" t="n">
+        <v>1.516911077624158</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1.578611598936505</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
         <v>2025</v>
       </c>
       <c r="B17" t="n">
-        <v>1.381777781720776</v>
+        <v>1.371697604134962</v>
       </c>
       <c r="C17" t="n">
-        <v>1.485674454593312</v>
+        <v>1.459365435341912</v>
       </c>
       <c r="D17" t="n">
-        <v>1.589571127465848</v>
+        <v>1.547033266548862</v>
       </c>
       <c r="E17" t="n">
-        <v>1.66269348934704</v>
+        <v>1.608733787861209</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1.371697604134962</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1.459365435341912</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1.547033266548862</v>
+      </c>
+      <c r="K17" t="n">
+        <v>1.608733787861209</v>
       </c>
     </row>
     <row r="18">
@@ -732,16 +1050,34 @@
         <v>2026</v>
       </c>
       <c r="B18" t="n">
-        <v>1.41626737489441</v>
+        <v>1.40121321292369</v>
       </c>
       <c r="C18" t="n">
-        <v>1.522569559201628</v>
+        <v>1.488881044569065</v>
       </c>
       <c r="D18" t="n">
-        <v>1.628871743508846</v>
+        <v>1.57654887621444</v>
       </c>
       <c r="E18" t="n">
-        <v>1.703687101640764</v>
+        <v>1.63824939783535</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1.40121321292369</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1.488881044569065</v>
+      </c>
+      <c r="J18" t="n">
+        <v>1.57654887621444</v>
+      </c>
+      <c r="K18" t="n">
+        <v>1.63824939783535</v>
       </c>
     </row>
     <row r="19">
@@ -749,16 +1085,34 @@
         <v>2027</v>
       </c>
       <c r="B19" t="n">
-        <v>1.450536878348918</v>
+        <v>1.430138509527791</v>
       </c>
       <c r="C19" t="n">
-        <v>1.559464663809944</v>
+        <v>1.517806341611675</v>
       </c>
       <c r="D19" t="n">
-        <v>1.66839244927097</v>
+        <v>1.605474173695559</v>
       </c>
       <c r="E19" t="n">
-        <v>1.745055702551176</v>
+        <v>1.667174695625092</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1.430138509527791</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1.517806341611675</v>
+      </c>
+      <c r="J19" t="n">
+        <v>1.605474173695559</v>
+      </c>
+      <c r="K19" t="n">
+        <v>1.667174695625092</v>
       </c>
     </row>
     <row r="20">
@@ -766,16 +1120,34 @@
         <v>2028</v>
       </c>
       <c r="B20" t="n">
-        <v>1.484601800270446</v>
+        <v>1.458485300190957</v>
       </c>
       <c r="C20" t="n">
-        <v>1.59635976841826</v>
+        <v>1.546153132713433</v>
       </c>
       <c r="D20" t="n">
-        <v>1.708117736566074</v>
+        <v>1.633820965235909</v>
       </c>
       <c r="E20" t="n">
-        <v>1.786772869248108</v>
+        <v>1.695521487474122</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1.458485300190957</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1.546153132713433</v>
+      </c>
+      <c r="J20" t="n">
+        <v>1.633820965235909</v>
+      </c>
+      <c r="K20" t="n">
+        <v>1.695521487474122</v>
       </c>
     </row>
     <row r="21">
@@ -783,16 +1155,34 @@
         <v>2029</v>
       </c>
       <c r="B21" t="n">
-        <v>1.518477270571168</v>
+        <v>1.486265155032007</v>
       </c>
       <c r="C21" t="n">
-        <v>1.633254873026576</v>
+        <v>1.573932987993156</v>
       </c>
       <c r="D21" t="n">
-        <v>1.748032475481984</v>
+        <v>1.661600820954304</v>
       </c>
       <c r="E21" t="n">
-        <v>1.828812823404159</v>
+        <v>1.723301343501254</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1.486265155032007</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1.573932987993156</v>
+      </c>
+      <c r="J21" t="n">
+        <v>1.661600820954304</v>
+      </c>
+      <c r="K21" t="n">
+        <v>1.723301343501254</v>
       </c>
     </row>
     <row r="22">
@@ -800,16 +1190,34 @@
         <v>2030</v>
       </c>
       <c r="B22" t="n">
-        <v>1.552177833347492</v>
+        <v>1.513489412767383</v>
       </c>
       <c r="C22" t="n">
-        <v>1.670149977634892</v>
+        <v>1.601157246167284</v>
       </c>
       <c r="D22" t="n">
-        <v>1.788122121922292</v>
+        <v>1.688825079567184</v>
       </c>
       <c r="E22" t="n">
-        <v>1.871150784804179</v>
+        <v>1.750525602422928</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1.513489412767383</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1.601157246167284</v>
+      </c>
+      <c r="J22" t="n">
+        <v>1.688825079567184</v>
+      </c>
+      <c r="K22" t="n">
+        <v>1.750525602422928</v>
       </c>
     </row>
     <row r="23">
@@ -817,16 +1225,34 @@
         <v>2031</v>
       </c>
       <c r="B23" t="n">
-        <v>1.58571730104176</v>
+        <v>1.540169185339199</v>
       </c>
       <c r="C23" t="n">
-        <v>1.707045082243208</v>
+        <v>1.627837019177929</v>
       </c>
       <c r="D23" t="n">
-        <v>1.828372863444657</v>
+        <v>1.71550485301666</v>
       </c>
       <c r="E23" t="n">
-        <v>1.91376321982439</v>
+        <v>1.777205376181251</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1.540169185339199</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1.627837019177929</v>
+      </c>
+      <c r="J23" t="n">
+        <v>1.71550485301666</v>
+      </c>
+      <c r="K23" t="n">
+        <v>1.777205376181251</v>
       </c>
     </row>
     <row r="24">
@@ -834,16 +1260,34 @@
         <v>2032</v>
       </c>
       <c r="B24" t="n">
-        <v>1.61910866176438</v>
+        <v>1.566315362450726</v>
       </c>
       <c r="C24" t="n">
-        <v>1.743940186851524</v>
+        <v>1.653983196728362</v>
       </c>
       <c r="D24" t="n">
-        <v>1.868771711938669</v>
+        <v>1.741651031005998</v>
       </c>
       <c r="E24" t="n">
-        <v>1.95662799933684</v>
+        <v>1.803351554479491</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1.566315362450726</v>
+      </c>
+      <c r="I24" t="n">
+        <v>1.653983196728362</v>
+      </c>
+      <c r="J24" t="n">
+        <v>1.741651031005998</v>
+      </c>
+      <c r="K24" t="n">
+        <v>1.803351554479491</v>
       </c>
     </row>
     <row r="25">
@@ -851,16 +1295,34 @@
         <v>2033</v>
       </c>
       <c r="B25" t="n">
-        <v>1.652364030236223</v>
+        <v>1.59193861601117</v>
       </c>
       <c r="C25" t="n">
-        <v>1.78083529145984</v>
+        <v>1.679606450727786</v>
       </c>
       <c r="D25" t="n">
-        <v>1.909306552683457</v>
+        <v>1.767274285444403</v>
       </c>
       <c r="E25" t="n">
-        <v>1.999724482293692</v>
+        <v>1.828974809226849</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="n">
+        <v>1.59193861601117</v>
+      </c>
+      <c r="I25" t="n">
+        <v>1.679606450727786</v>
+      </c>
+      <c r="J25" t="n">
+        <v>1.767274285444403</v>
+      </c>
+      <c r="K25" t="n">
+        <v>1.828974809226849</v>
       </c>
     </row>
     <row r="26">
@@ -868,16 +1330,34 @@
         <v>2034</v>
       </c>
       <c r="B26" t="n">
-        <v>1.685494632957898</v>
+        <v>1.617049404491552</v>
       </c>
       <c r="C26" t="n">
-        <v>1.817730396068156</v>
+        <v>1.704717239647222</v>
       </c>
       <c r="D26" t="n">
-        <v>1.949966159178415</v>
+        <v>1.792385074802892</v>
       </c>
       <c r="E26" t="n">
-        <v>2.043033540995796</v>
+        <v>1.854085598894344</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="n">
+        <v>1.617049404491552</v>
+      </c>
+      <c r="I26" t="n">
+        <v>1.704717239647222</v>
+      </c>
+      <c r="J26" t="n">
+        <v>1.792385074802892</v>
+      </c>
+      <c r="K26" t="n">
+        <v>1.854085598894344</v>
       </c>
     </row>
     <row r="27">
@@ -885,16 +1365,34 @@
         <v>2035</v>
       </c>
       <c r="B27" t="n">
-        <v>1.718510819065151</v>
+        <v>1.641657977193473</v>
       </c>
       <c r="C27" t="n">
-        <v>1.854625500676472</v>
+        <v>1.729325812788269</v>
       </c>
       <c r="D27" t="n">
-        <v>1.990740182287793</v>
+        <v>1.816993648383064</v>
       </c>
       <c r="E27" t="n">
-        <v>2.086537542597271</v>
+        <v>1.878694172783572</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1.641657977193473</v>
+      </c>
+      <c r="I27" t="n">
+        <v>1.729325812788269</v>
+      </c>
+      <c r="J27" t="n">
+        <v>1.816993648383064</v>
+      </c>
+      <c r="K27" t="n">
+        <v>1.878694172783572</v>
       </c>
     </row>
     <row r="28">
@@ -902,16 +1400,34 @@
         <v>2036</v>
       </c>
       <c r="B28" t="n">
-        <v>1.75142208953799</v>
+        <v>1.665774378432503</v>
       </c>
       <c r="C28" t="n">
-        <v>1.891520605284788</v>
+        <v>1.753442214466495</v>
       </c>
       <c r="D28" t="n">
-        <v>2.031619121031587</v>
+        <v>1.841110050500486</v>
       </c>
       <c r="E28" t="n">
-        <v>2.130220299339032</v>
+        <v>1.902810575210099</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" t="n">
+        <v>1.665774378432503</v>
+      </c>
+      <c r="I28" t="n">
+        <v>1.753442214466495</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1.841110050500486</v>
+      </c>
+      <c r="K28" t="n">
+        <v>1.902810575210099</v>
       </c>
     </row>
     <row r="29">
@@ -919,16 +1435,34 @@
         <v>2037</v>
       </c>
       <c r="B29" t="n">
-        <v>1.784237138746285</v>
+        <v>1.6894084516379</v>
       </c>
       <c r="C29" t="n">
-        <v>1.928415709893105</v>
+        <v>1.777076288111156</v>
       </c>
       <c r="D29" t="n">
-        <v>2.072594281039924</v>
+        <v>1.864744124584411</v>
       </c>
       <c r="E29" t="n">
-        <v>2.174066997763443</v>
+        <v>1.926444649603178</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" t="n">
+        <v>1.6894084516379</v>
+      </c>
+      <c r="I29" t="n">
+        <v>1.777076288111156</v>
+      </c>
+      <c r="J29" t="n">
+        <v>1.864744124584411</v>
+      </c>
+      <c r="K29" t="n">
+        <v>1.926444649603178</v>
       </c>
     </row>
     <row r="30">
@@ -936,16 +1470,34 @@
         <v>2038</v>
       </c>
       <c r="B30" t="n">
-        <v>1.816963903578842</v>
+        <v>1.712569843370337</v>
       </c>
       <c r="C30" t="n">
-        <v>1.96531081450142</v>
+        <v>1.800237680282924</v>
       </c>
       <c r="D30" t="n">
-        <v>2.113657725423999</v>
+        <v>1.887905517195511</v>
       </c>
       <c r="E30" t="n">
-        <v>2.218064115008253</v>
+        <v>1.94960604252348</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" t="n">
+        <v>1.712569843370337</v>
+      </c>
+      <c r="I30" t="n">
+        <v>1.800237680282924</v>
+      </c>
+      <c r="J30" t="n">
+        <v>1.887905517195511</v>
+      </c>
+      <c r="K30" t="n">
+        <v>1.94960604252348</v>
       </c>
     </row>
     <row r="31">
@@ -953,16 +1505,34 @@
         <v>2039</v>
       </c>
       <c r="B31" t="n">
-        <v>1.849609616529605</v>
+        <v>1.735268007259272</v>
       </c>
       <c r="C31" t="n">
-        <v>2.002205919109736</v>
+        <v>1.822935844611257</v>
       </c>
       <c r="D31" t="n">
-        <v>2.154802221689868</v>
+        <v>1.910603681963242</v>
       </c>
       <c r="E31" t="n">
-        <v>2.262199328358391</v>
+        <v>1.972304207600458</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" t="n">
+        <v>1.735268007259272</v>
+      </c>
+      <c r="I31" t="n">
+        <v>1.822935844611257</v>
+      </c>
+      <c r="J31" t="n">
+        <v>1.910603681963242</v>
+      </c>
+      <c r="K31" t="n">
+        <v>1.972304207600458</v>
       </c>
     </row>
     <row r="32">
@@ -970,16 +1540,34 @@
         <v>2040</v>
       </c>
       <c r="B32" t="n">
-        <v>1.882180860067304</v>
+        <v>1.757512207861575</v>
       </c>
       <c r="C32" t="n">
-        <v>2.039101023718052</v>
+        <v>1.845180045653023</v>
       </c>
       <c r="D32" t="n">
-        <v>2.196021187368801</v>
+        <v>1.932847883444471</v>
       </c>
       <c r="E32" t="n">
-        <v>2.306461422611013</v>
+        <v>1.994548409390981</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" t="n">
+        <v>1.757512207861575</v>
+      </c>
+      <c r="I32" t="n">
+        <v>1.845180045653023</v>
+      </c>
+      <c r="J32" t="n">
+        <v>1.932847883444471</v>
+      </c>
+      <c r="K32" t="n">
+        <v>1.994548409390981</v>
       </c>
     </row>
     <row r="33">
@@ -987,16 +1575,34 @@
         <v>2041</v>
       </c>
       <c r="B33" t="n">
-        <v>1.914683620388837</v>
+        <v>1.779311524442979</v>
       </c>
       <c r="C33" t="n">
-        <v>2.075996128326369</v>
+        <v>1.866979362673954</v>
       </c>
       <c r="D33" t="n">
-        <v>2.237308636263899</v>
+        <v>1.954647200904928</v>
       </c>
       <c r="E33" t="n">
-        <v>2.350840198490556</v>
+        <v>2.016347727160776</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" t="n">
+        <v>1.779311524442979</v>
+      </c>
+      <c r="I33" t="n">
+        <v>1.866979362673954</v>
+      </c>
+      <c r="J33" t="n">
+        <v>1.954647200904928</v>
+      </c>
+      <c r="K33" t="n">
+        <v>2.016347727160776</v>
       </c>
     </row>
     <row r="34">
@@ -1004,16 +1610,34 @@
         <v>2042</v>
       </c>
       <c r="B34" t="n">
-        <v>1.947123339265392</v>
+        <v>1.800674854683903</v>
       </c>
       <c r="C34" t="n">
-        <v>2.112891232934685</v>
+        <v>1.888342693354466</v>
       </c>
       <c r="D34" t="n">
-        <v>2.278659126603977</v>
+        <v>1.976010532025029</v>
       </c>
       <c r="E34" t="n">
-        <v>2.395326384313374</v>
+        <v>2.037711058590259</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" t="n">
+        <v>1.800674854683903</v>
+      </c>
+      <c r="I34" t="n">
+        <v>1.888342693354466</v>
+      </c>
+      <c r="J34" t="n">
+        <v>1.976010532025029</v>
+      </c>
+      <c r="K34" t="n">
+        <v>2.037711058590259</v>
       </c>
     </row>
     <row r="35">
@@ -1021,16 +1645,34 @@
         <v>2043</v>
       </c>
       <c r="B35" t="n">
-        <v>1.979504963155712</v>
+        <v>1.821610918311155</v>
       </c>
       <c r="C35" t="n">
-        <v>2.149786337543001</v>
+        <v>1.909278757421368</v>
       </c>
       <c r="D35" t="n">
-        <v>2.320067711930289</v>
+        <v>1.996946596531581</v>
       </c>
       <c r="E35" t="n">
-        <v>2.439911552308603</v>
+        <v>2.058647123406236</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" t="n">
+        <v>1.821610918311155</v>
+      </c>
+      <c r="I35" t="n">
+        <v>1.909278757421368</v>
+      </c>
+      <c r="J35" t="n">
+        <v>1.996946596531581</v>
+      </c>
+      <c r="K35" t="n">
+        <v>2.058647123406236</v>
       </c>
     </row>
     <row r="36">
@@ -1038,16 +1680,34 @@
         <v>2044</v>
       </c>
       <c r="B36" t="n">
-        <v>2.011832989107607</v>
+        <v>1.842128260657009</v>
       </c>
       <c r="C36" t="n">
-        <v>2.186681442151317</v>
+        <v>1.929796100206932</v>
       </c>
       <c r="D36" t="n">
-        <v>2.361529895195027</v>
+        <v>2.017463939756855</v>
       </c>
       <c r="E36" t="n">
-        <v>2.484588040411228</v>
+        <v>2.079164466940977</v>
+      </c>
+      <c r="F36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" t="n">
+        <v>1.842128260657009</v>
+      </c>
+      <c r="I36" t="n">
+        <v>1.929796100206932</v>
+      </c>
+      <c r="J36" t="n">
+        <v>2.017463939756855</v>
+      </c>
+      <c r="K36" t="n">
+        <v>2.079164466940977</v>
       </c>
     </row>
     <row r="37">
@@ -1055,16 +1715,34 @@
         <v>2045</v>
       </c>
       <c r="B37" t="n">
-        <v>2.044111507220202</v>
+        <v>1.862235256147094</v>
       </c>
       <c r="C37" t="n">
-        <v>2.223576546759633</v>
+        <v>1.949903096136785</v>
       </c>
       <c r="D37" t="n">
-        <v>2.403041586299064</v>
+        <v>2.037570936126476</v>
       </c>
       <c r="E37" t="n">
-        <v>2.529348879914946</v>
+        <v>2.099271463620106</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" t="n">
+        <v>1.862235256147094</v>
+      </c>
+      <c r="I37" t="n">
+        <v>1.949903096136785</v>
+      </c>
+      <c r="J37" t="n">
+        <v>2.037570936126476</v>
+      </c>
+      <c r="K37" t="n">
+        <v>2.099271463620106</v>
       </c>
     </row>
     <row r="38">
@@ -1072,16 +1750,34 @@
         <v>2046</v>
       </c>
       <c r="B38" t="n">
-        <v>2.076344239616657</v>
+        <v>1.881940111718524</v>
       </c>
       <c r="C38" t="n">
-        <v>2.260471651367949</v>
+        <v>1.969607952148041</v>
       </c>
       <c r="D38" t="n">
-        <v>2.444599063119241</v>
+        <v>2.057275792577557</v>
       </c>
       <c r="E38" t="n">
-        <v>2.574187729070489</v>
+        <v>2.118976320380736</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" t="n">
+        <v>1.881940111718524</v>
+      </c>
+      <c r="I38" t="n">
+        <v>1.969607952148041</v>
+      </c>
+      <c r="J38" t="n">
+        <v>2.057275792577557</v>
+      </c>
+      <c r="K38" t="n">
+        <v>2.118976320380736</v>
       </c>
     </row>
     <row r="39">
@@ -1089,16 +1785,34 @@
         <v>2047</v>
       </c>
       <c r="B39" t="n">
-        <v>2.108534575997663</v>
+        <v>1.901250870169673</v>
       </c>
       <c r="C39" t="n">
-        <v>2.297366755976265</v>
+        <v>1.988918711039071</v>
       </c>
       <c r="D39" t="n">
-        <v>2.486198935954867</v>
+        <v>2.076586551908469</v>
       </c>
       <c r="E39" t="n">
-        <v>2.619098812509622</v>
+        <v>2.138287080021236</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" t="n">
+        <v>1.901250870169673</v>
+      </c>
+      <c r="I39" t="n">
+        <v>1.988918711039071</v>
+      </c>
+      <c r="J39" t="n">
+        <v>2.076586551908469</v>
+      </c>
+      <c r="K39" t="n">
+        <v>2.138287080021236</v>
       </c>
     </row>
     <row r="40">
@@ -1106,16 +1820,34 @@
         <v>2048</v>
       </c>
       <c r="B40" t="n">
-        <v>2.14068560592434</v>
+        <v>1.920175413442945</v>
       </c>
       <c r="C40" t="n">
-        <v>2.334261860584581</v>
+        <v>2.007843254752281</v>
       </c>
       <c r="D40" t="n">
-        <v>2.527838115244823</v>
+        <v>2.095511096061616</v>
       </c>
       <c r="E40" t="n">
-        <v>2.664076866241571</v>
+        <v>2.15721162448401</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" t="n">
+        <v>1.920175413442945</v>
+      </c>
+      <c r="I40" t="n">
+        <v>2.007843254752281</v>
+      </c>
+      <c r="J40" t="n">
+        <v>2.095511096061616</v>
+      </c>
+      <c r="K40" t="n">
+        <v>2.15721162448401</v>
       </c>
     </row>
     <row r="41">
@@ -1123,16 +1855,34 @@
         <v>2049</v>
       </c>
       <c r="B41" t="n">
-        <v>2.172800148026589</v>
+        <v>1.9387214658419</v>
       </c>
       <c r="C41" t="n">
-        <v>2.371156965192897</v>
+        <v>2.026389307591226</v>
       </c>
       <c r="D41" t="n">
-        <v>2.569513782359206</v>
+        <v>2.114057149340553</v>
       </c>
       <c r="E41" t="n">
-        <v>2.709117087887869</v>
+        <v>2.175757678072613</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" t="n">
+        <v>1</v>
+      </c>
+      <c r="H41" t="n">
+        <v>1.9387214658419</v>
+      </c>
+      <c r="I41" t="n">
+        <v>2.026389307591226</v>
+      </c>
+      <c r="J41" t="n">
+        <v>2.114057149340553</v>
+      </c>
+      <c r="K41" t="n">
+        <v>2.175757678072613</v>
       </c>
     </row>
     <row r="42">
@@ -1140,16 +1890,34 @@
         <v>2050</v>
       </c>
       <c r="B42" t="n">
-        <v>2.204880776358147</v>
+        <v>1.956896597184022</v>
       </c>
       <c r="C42" t="n">
-        <v>2.408052069801213</v>
+        <v>2.044564439373393</v>
       </c>
       <c r="D42" t="n">
-        <v>2.611223363244279</v>
+        <v>2.132232281562764</v>
       </c>
       <c r="E42" t="n">
-        <v>2.754215091778648</v>
+        <v>2.193932810604526</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" t="n">
+        <v>1.956896597184022</v>
+      </c>
+      <c r="I42" t="n">
+        <v>2.044564439373393</v>
+      </c>
+      <c r="J42" t="n">
+        <v>2.132232281562764</v>
+      </c>
+      <c r="K42" t="n">
+        <v>2.193932810604526</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Paper4 tolerance tasks and Ag2050 labor workflows
</commit_message>
<xml_diff>
--- a/myCode/Ag2050/2_processed_data/labour_cost_forecast.xlsx
+++ b/myCode/Ag2050/2_processed_data/labour_cost_forecast.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="fitted_scenarios" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="actual_history" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="growth_rate_method" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -491,22 +492,22 @@
         <v>2010</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8493209550512516</v>
+        <v>0.9791920419343512</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9369887862582014</v>
+        <v>0.9791920419343512</v>
       </c>
       <c r="D2" t="n">
-        <v>1.024656617465151</v>
+        <v>0.9791920419343512</v>
       </c>
       <c r="E2" t="n">
-        <v>1.086357138777498</v>
+        <v>0.9791920419343512</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9369887862582014</v>
+        <v>0.9791920419343512</v>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
@@ -518,22 +519,22 @@
         <v>2011</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8892904903072976</v>
+        <v>1.019161577190397</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9769583215142472</v>
+        <v>1.019161577190397</v>
       </c>
       <c r="D3" t="n">
-        <v>1.064626152721197</v>
+        <v>1.019161577190397</v>
       </c>
       <c r="E3" t="n">
-        <v>1.126326674033544</v>
+        <v>1.019161577190397</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9769583215142472</v>
+        <v>1.019161577190397</v>
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
@@ -545,22 +546,22 @@
         <v>2012</v>
       </c>
       <c r="B4" t="n">
-        <v>0.9284567641529331</v>
+        <v>1.058327851036033</v>
       </c>
       <c r="C4" t="n">
-        <v>1.016124595359883</v>
+        <v>1.058327851036033</v>
       </c>
       <c r="D4" t="n">
-        <v>1.103792426566833</v>
+        <v>1.058327851036033</v>
       </c>
       <c r="E4" t="n">
-        <v>1.16549294787918</v>
+        <v>1.058327851036033</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>1.016124595359883</v>
+        <v>1.058327851036033</v>
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
@@ -572,22 +573,22 @@
         <v>2013</v>
       </c>
       <c r="B5" t="n">
-        <v>0.9668358418196071</v>
+        <v>1.096706928702707</v>
       </c>
       <c r="C5" t="n">
-        <v>1.054503673026557</v>
+        <v>1.096706928702707</v>
       </c>
       <c r="D5" t="n">
-        <v>1.142171504233507</v>
+        <v>1.096706928702707</v>
       </c>
       <c r="E5" t="n">
-        <v>1.203872025545853</v>
+        <v>1.096706928702707</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>1.054503673026557</v>
+        <v>1.096706928702707</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
@@ -599,22 +600,22 @@
         <v>2014</v>
       </c>
       <c r="B6" t="n">
-        <v>1.004443467241855</v>
+        <v>1.134314554124954</v>
       </c>
       <c r="C6" t="n">
-        <v>1.092111298448804</v>
+        <v>1.134314554124954</v>
       </c>
       <c r="D6" t="n">
-        <v>1.179779129655754</v>
+        <v>1.134314554124954</v>
       </c>
       <c r="E6" t="n">
-        <v>1.241479650968101</v>
+        <v>1.134314554124954</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>1.092111298448804</v>
+        <v>1.134314554124954</v>
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
@@ -626,22 +627,22 @@
         <v>2015</v>
       </c>
       <c r="B7" t="n">
-        <v>1.041295069483078</v>
+        <v>1.171166156366177</v>
       </c>
       <c r="C7" t="n">
-        <v>1.128962900690027</v>
+        <v>1.171166156366177</v>
       </c>
       <c r="D7" t="n">
-        <v>1.216630731896977</v>
+        <v>1.171166156366177</v>
       </c>
       <c r="E7" t="n">
-        <v>1.278331253209324</v>
+        <v>1.171166156366177</v>
       </c>
       <c r="F7" t="n">
         <v>1.153908543682574</v>
       </c>
       <c r="G7" t="n">
-        <v>1.128962900690027</v>
+        <v>1.171166156366177</v>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
@@ -653,22 +654,22 @@
         <v>2016</v>
       </c>
       <c r="B8" t="n">
-        <v>1.077421161395491</v>
+        <v>1.207292248278591</v>
       </c>
       <c r="C8" t="n">
-        <v>1.165088992602441</v>
+        <v>1.207292248278591</v>
       </c>
       <c r="D8" t="n">
-        <v>1.25275682380939</v>
+        <v>1.207292248278591</v>
       </c>
       <c r="E8" t="n">
-        <v>1.314457345121738</v>
+        <v>1.207292248278591</v>
       </c>
       <c r="F8" t="n">
         <v>1.14257096572451</v>
       </c>
       <c r="G8" t="n">
-        <v>1.165088992602441</v>
+        <v>1.207292248278591</v>
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
@@ -680,22 +681,22 @@
         <v>2017</v>
       </c>
       <c r="B9" t="n">
-        <v>1.112820034773279</v>
+        <v>1.242691121656378</v>
       </c>
       <c r="C9" t="n">
-        <v>1.200487865980228</v>
+        <v>1.242691121656378</v>
       </c>
       <c r="D9" t="n">
-        <v>1.288155697187178</v>
+        <v>1.242691121656378</v>
       </c>
       <c r="E9" t="n">
-        <v>1.349856218499525</v>
+        <v>1.242691121656378</v>
       </c>
       <c r="F9" t="n">
         <v>1.208048138561229</v>
       </c>
       <c r="G9" t="n">
-        <v>1.200487865980228</v>
+        <v>1.242691121656378</v>
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
@@ -707,22 +708,22 @@
         <v>2018</v>
       </c>
       <c r="B10" t="n">
-        <v>1.147513893551493</v>
+        <v>1.277384980434593</v>
       </c>
       <c r="C10" t="n">
-        <v>1.235181724758443</v>
+        <v>1.277384980434593</v>
       </c>
       <c r="D10" t="n">
-        <v>1.322849555965392</v>
+        <v>1.277384980434593</v>
       </c>
       <c r="E10" t="n">
-        <v>1.384550077277739</v>
+        <v>1.277384980434593</v>
       </c>
       <c r="F10" t="n">
         <v>1.215777713114327</v>
       </c>
       <c r="G10" t="n">
-        <v>1.235181724758443</v>
+        <v>1.277384980434593</v>
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
@@ -734,22 +735,22 @@
         <v>2019</v>
       </c>
       <c r="B11" t="n">
-        <v>1.181511193656107</v>
+        <v>1.311382280539206</v>
       </c>
       <c r="C11" t="n">
-        <v>1.269179024863056</v>
+        <v>1.311382280539206</v>
       </c>
       <c r="D11" t="n">
-        <v>1.356846856070006</v>
+        <v>1.311382280539206</v>
       </c>
       <c r="E11" t="n">
-        <v>1.418547377382353</v>
+        <v>1.311382280539206</v>
       </c>
       <c r="F11" t="n">
         <v>1.358509372339871</v>
       </c>
       <c r="G11" t="n">
-        <v>1.269179024863056</v>
+        <v>1.311382280539206</v>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
@@ -761,22 +762,22 @@
         <v>2020</v>
       </c>
       <c r="B12" t="n">
-        <v>1.214839383261954</v>
+        <v>1.344710470145054</v>
       </c>
       <c r="C12" t="n">
-        <v>1.302507214468904</v>
+        <v>1.344710470145054</v>
       </c>
       <c r="D12" t="n">
-        <v>1.390175045675853</v>
+        <v>1.344710470145054</v>
       </c>
       <c r="E12" t="n">
-        <v>1.451875566988201</v>
+        <v>1.344710470145054</v>
       </c>
       <c r="F12" t="n">
         <v>1.105484425759602</v>
       </c>
       <c r="G12" t="n">
-        <v>1.302507214468904</v>
+        <v>1.344710470145054</v>
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
@@ -788,22 +789,22 @@
         <v>2021</v>
       </c>
       <c r="B13" t="n">
-        <v>1.247472550491938</v>
+        <v>1.377343637375037</v>
       </c>
       <c r="C13" t="n">
-        <v>1.335140381698887</v>
+        <v>1.377343637375037</v>
       </c>
       <c r="D13" t="n">
-        <v>1.422808212905837</v>
+        <v>1.377343637375037</v>
       </c>
       <c r="E13" t="n">
-        <v>1.484508734218184</v>
+        <v>1.377343637375037</v>
       </c>
       <c r="F13" t="n">
         <v>1.276148524225631</v>
       </c>
       <c r="G13" t="n">
-        <v>1.335140381698887</v>
+        <v>1.377343637375037</v>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
@@ -815,22 +816,22 @@
         <v>2022</v>
       </c>
       <c r="B14" t="n">
-        <v>1.279466462846748</v>
+        <v>1.409337549729847</v>
       </c>
       <c r="C14" t="n">
-        <v>1.367134294053697</v>
+        <v>1.409337549729847</v>
       </c>
       <c r="D14" t="n">
-        <v>1.454802125260647</v>
+        <v>1.409337549729847</v>
       </c>
       <c r="E14" t="n">
-        <v>1.516502646572994</v>
+        <v>1.409337549729847</v>
       </c>
       <c r="F14" t="n">
         <v>1.49238768827198</v>
       </c>
       <c r="G14" t="n">
-        <v>1.367134294053697</v>
+        <v>1.409337549729847</v>
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
@@ -842,22 +843,22 @@
         <v>2023</v>
       </c>
       <c r="B15" t="n">
-        <v>1.310838804723399</v>
+        <v>1.440709891606498</v>
       </c>
       <c r="C15" t="n">
-        <v>1.398506635930348</v>
+        <v>1.440709891606498</v>
       </c>
       <c r="D15" t="n">
-        <v>1.486174467137298</v>
+        <v>1.440709891606498</v>
       </c>
       <c r="E15" t="n">
-        <v>1.547874988449645</v>
+        <v>1.440709891606498</v>
       </c>
       <c r="F15" t="n">
         <v>1.438405529593662</v>
       </c>
       <c r="G15" t="n">
-        <v>1.398506635930348</v>
+        <v>1.440709891606498</v>
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
@@ -869,34 +870,34 @@
         <v>2024</v>
       </c>
       <c r="B16" t="n">
-        <v>1.341575415210259</v>
+        <v>1.471446502093358</v>
       </c>
       <c r="C16" t="n">
-        <v>1.429243246417209</v>
+        <v>1.471446502093358</v>
       </c>
       <c r="D16" t="n">
-        <v>1.516911077624158</v>
+        <v>1.471446502093358</v>
       </c>
       <c r="E16" t="n">
-        <v>1.578611598936505</v>
+        <v>1.471446502093358</v>
       </c>
       <c r="F16" t="n">
         <v>1.471446502093358</v>
       </c>
       <c r="G16" t="n">
-        <v>1.429243246417209</v>
+        <v>1.471446502093358</v>
       </c>
       <c r="H16" t="n">
-        <v>1.341575415210259</v>
+        <v>1.471446502093358</v>
       </c>
       <c r="I16" t="n">
-        <v>1.429243246417209</v>
+        <v>1.471446502093358</v>
       </c>
       <c r="J16" t="n">
-        <v>1.516911077624158</v>
+        <v>1.471446502093358</v>
       </c>
       <c r="K16" t="n">
-        <v>1.578611598936505</v>
+        <v>1.471446502093358</v>
       </c>
     </row>
     <row r="17">
@@ -904,30 +905,30 @@
         <v>2025</v>
       </c>
       <c r="B17" t="n">
-        <v>1.371697604134962</v>
+        <v>1.486431296108713</v>
       </c>
       <c r="C17" t="n">
-        <v>1.459365435341912</v>
+        <v>1.501568691018062</v>
       </c>
       <c r="D17" t="n">
-        <v>1.547033266548862</v>
+        <v>1.516860240865645</v>
       </c>
       <c r="E17" t="n">
-        <v>1.608733787861209</v>
+        <v>1.532307515521649</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>1.371697604134962</v>
+        <v>1.486431296108713</v>
       </c>
       <c r="I17" t="n">
-        <v>1.459365435341912</v>
+        <v>1.501568691018062</v>
       </c>
       <c r="J17" t="n">
-        <v>1.547033266548862</v>
+        <v>1.516860240865645</v>
       </c>
       <c r="K17" t="n">
-        <v>1.608733787861209</v>
+        <v>1.532307515521649</v>
       </c>
     </row>
     <row r="18">
@@ -935,30 +936,30 @@
         <v>2026</v>
       </c>
       <c r="B18" t="n">
-        <v>1.40121321292369</v>
+        <v>1.500969232864511</v>
       </c>
       <c r="C18" t="n">
-        <v>1.488881044569065</v>
+        <v>1.531084300245215</v>
       </c>
       <c r="D18" t="n">
-        <v>1.57654887621444</v>
+        <v>1.561803588727516</v>
       </c>
       <c r="E18" t="n">
-        <v>1.63824939783535</v>
+        <v>1.593139221250904</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>1.40121321292369</v>
+        <v>1.500969232864511</v>
       </c>
       <c r="I18" t="n">
-        <v>1.488881044569065</v>
+        <v>1.531084300245215</v>
       </c>
       <c r="J18" t="n">
-        <v>1.57654887621444</v>
+        <v>1.561803588727516</v>
       </c>
       <c r="K18" t="n">
-        <v>1.63824939783535</v>
+        <v>1.593139221250904</v>
       </c>
     </row>
     <row r="19">
@@ -966,30 +967,30 @@
         <v>2027</v>
       </c>
       <c r="B19" t="n">
-        <v>1.430138509527791</v>
+        <v>1.515081075441588</v>
       </c>
       <c r="C19" t="n">
-        <v>1.517806341611675</v>
+        <v>1.560009597287825</v>
       </c>
       <c r="D19" t="n">
-        <v>1.605474173695559</v>
+        <v>1.606270438643564</v>
       </c>
       <c r="E19" t="n">
-        <v>1.667174695625092</v>
+        <v>1.653903108382065</v>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>1.430138509527791</v>
+        <v>1.515081075441588</v>
       </c>
       <c r="I19" t="n">
-        <v>1.517806341611675</v>
+        <v>1.560009597287825</v>
       </c>
       <c r="J19" t="n">
-        <v>1.605474173695559</v>
+        <v>1.606270438643564</v>
       </c>
       <c r="K19" t="n">
-        <v>1.667174695625092</v>
+        <v>1.653903108382065</v>
       </c>
     </row>
     <row r="20">
@@ -997,30 +998,30 @@
         <v>2028</v>
       </c>
       <c r="B20" t="n">
-        <v>1.458485300190957</v>
+        <v>1.528784305182877</v>
       </c>
       <c r="C20" t="n">
-        <v>1.546153132713433</v>
+        <v>1.588356388389583</v>
       </c>
       <c r="D20" t="n">
-        <v>1.633820965235909</v>
+        <v>1.650249814826694</v>
       </c>
       <c r="E20" t="n">
-        <v>1.695521487474122</v>
+        <v>1.714555040192641</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>1.458485300190957</v>
+        <v>1.528784305182877</v>
       </c>
       <c r="I20" t="n">
-        <v>1.546153132713433</v>
+        <v>1.588356388389583</v>
       </c>
       <c r="J20" t="n">
-        <v>1.633820965235909</v>
+        <v>1.650249814826694</v>
       </c>
       <c r="K20" t="n">
-        <v>1.695521487474122</v>
+        <v>1.714555040192641</v>
       </c>
     </row>
     <row r="21">
@@ -1028,30 +1029,30 @@
         <v>2029</v>
       </c>
       <c r="B21" t="n">
-        <v>1.486265155032007</v>
+        <v>1.542095335137714</v>
       </c>
       <c r="C21" t="n">
-        <v>1.573932987993156</v>
+        <v>1.616136243669305</v>
       </c>
       <c r="D21" t="n">
-        <v>1.661600820954304</v>
+        <v>1.693732092035854</v>
       </c>
       <c r="E21" t="n">
-        <v>1.723301343501254</v>
+        <v>1.775053564221132</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>1.486265155032007</v>
+        <v>1.542095335137714</v>
       </c>
       <c r="I21" t="n">
-        <v>1.573932987993156</v>
+        <v>1.616136243669305</v>
       </c>
       <c r="J21" t="n">
-        <v>1.661600820954304</v>
+        <v>1.693732092035854</v>
       </c>
       <c r="K21" t="n">
-        <v>1.723301343501254</v>
+        <v>1.775053564221132</v>
       </c>
     </row>
     <row r="22">
@@ -1059,30 +1060,30 @@
         <v>2030</v>
       </c>
       <c r="B22" t="n">
-        <v>1.513489412767383</v>
+        <v>1.555029601684774</v>
       </c>
       <c r="C22" t="n">
-        <v>1.601157246167284</v>
+        <v>1.643360501843434</v>
       </c>
       <c r="D22" t="n">
-        <v>1.688825079567184</v>
+        <v>1.736708893575492</v>
       </c>
       <c r="E22" t="n">
-        <v>1.750525602422928</v>
+        <v>1.835359787241355</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>1.513489412767383</v>
+        <v>1.555029601684774</v>
       </c>
       <c r="I22" t="n">
-        <v>1.601157246167284</v>
+        <v>1.643360501843434</v>
       </c>
       <c r="J22" t="n">
-        <v>1.688825079567184</v>
+        <v>1.736708893575492</v>
       </c>
       <c r="K22" t="n">
-        <v>1.750525602422928</v>
+        <v>1.835359787241355</v>
       </c>
     </row>
     <row r="23">
@@ -1090,30 +1091,30 @@
         <v>2031</v>
       </c>
       <c r="B23" t="n">
-        <v>1.540169185339199</v>
+        <v>1.567601646078833</v>
       </c>
       <c r="C23" t="n">
-        <v>1.627837019177929</v>
+        <v>1.670040274854079</v>
       </c>
       <c r="D23" t="n">
-        <v>1.71550485301666</v>
+        <v>1.779172997560397</v>
       </c>
       <c r="E23" t="n">
-        <v>1.777205376181251</v>
+        <v>1.895437255562373</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>1.540169185339199</v>
+        <v>1.567601646078833</v>
       </c>
       <c r="I23" t="n">
-        <v>1.627837019177929</v>
+        <v>1.670040274854079</v>
       </c>
       <c r="J23" t="n">
-        <v>1.71550485301666</v>
+        <v>1.779172997560397</v>
       </c>
       <c r="K23" t="n">
-        <v>1.777205376181251</v>
+        <v>1.895437255562373</v>
       </c>
     </row>
     <row r="24">
@@ -1121,30 +1122,30 @@
         <v>2032</v>
       </c>
       <c r="B24" t="n">
-        <v>1.566315362450726</v>
+        <v>1.579825187256097</v>
       </c>
       <c r="C24" t="n">
-        <v>1.653983196728362</v>
+        <v>1.696186452404512</v>
       </c>
       <c r="D24" t="n">
-        <v>1.741651031005998</v>
+        <v>1.821118250632258</v>
       </c>
       <c r="E24" t="n">
-        <v>1.803351554479491</v>
+        <v>1.955251840435626</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>1.566315362450726</v>
+        <v>1.579825187256097</v>
       </c>
       <c r="I24" t="n">
-        <v>1.653983196728362</v>
+        <v>1.696186452404512</v>
       </c>
       <c r="J24" t="n">
-        <v>1.741651031005998</v>
+        <v>1.821118250632258</v>
       </c>
       <c r="K24" t="n">
-        <v>1.803351554479491</v>
+        <v>1.955251840435626</v>
       </c>
     </row>
     <row r="25">
@@ -1152,30 +1153,30 @@
         <v>2033</v>
       </c>
       <c r="B25" t="n">
-        <v>1.59193861601117</v>
+        <v>1.591713187027884</v>
       </c>
       <c r="C25" t="n">
-        <v>1.679606450727786</v>
+        <v>1.721809706403936</v>
       </c>
       <c r="D25" t="n">
-        <v>1.767274285444403</v>
+        <v>1.862539488412791</v>
       </c>
       <c r="E25" t="n">
-        <v>1.828974809226849</v>
+        <v>2.014771628359691</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>1.59193861601117</v>
+        <v>1.591713187027884</v>
       </c>
       <c r="I25" t="n">
-        <v>1.679606450727786</v>
+        <v>1.721809706403936</v>
       </c>
       <c r="J25" t="n">
-        <v>1.767274285444403</v>
+        <v>1.862539488412791</v>
       </c>
       <c r="K25" t="n">
-        <v>1.828974809226849</v>
+        <v>2.014771628359691</v>
       </c>
     </row>
     <row r="26">
@@ -1183,30 +1184,30 @@
         <v>2034</v>
       </c>
       <c r="B26" t="n">
-        <v>1.617049404491552</v>
+        <v>1.603277908623072</v>
       </c>
       <c r="C26" t="n">
-        <v>1.704717239647222</v>
+        <v>1.746920495323371</v>
       </c>
       <c r="D26" t="n">
-        <v>1.792385074802892</v>
+        <v>1.903432462062515</v>
       </c>
       <c r="E26" t="n">
-        <v>1.854085598894344</v>
+        <v>2.073966816081521</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>1.617049404491552</v>
+        <v>1.603277908623072</v>
       </c>
       <c r="I26" t="n">
-        <v>1.704717239647222</v>
+        <v>1.746920495323371</v>
       </c>
       <c r="J26" t="n">
-        <v>1.792385074802892</v>
+        <v>1.903432462062515</v>
       </c>
       <c r="K26" t="n">
-        <v>1.854085598894344</v>
+        <v>2.073966816081521</v>
       </c>
     </row>
     <row r="27">
@@ -1214,30 +1215,30 @@
         <v>2035</v>
       </c>
       <c r="B27" t="n">
-        <v>1.641657977193473</v>
+        <v>1.614530969399062</v>
       </c>
       <c r="C27" t="n">
-        <v>1.729325812788269</v>
+        <v>1.771529068464418</v>
       </c>
       <c r="D27" t="n">
-        <v>1.816993648383064</v>
+        <v>1.94379377038677</v>
       </c>
       <c r="E27" t="n">
-        <v>1.878694172783572</v>
+        <v>2.132809610101132</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>1.641657977193473</v>
+        <v>1.614530969399062</v>
       </c>
       <c r="I27" t="n">
-        <v>1.729325812788269</v>
+        <v>1.771529068464418</v>
       </c>
       <c r="J27" t="n">
-        <v>1.816993648383064</v>
+        <v>1.94379377038677</v>
       </c>
       <c r="K27" t="n">
-        <v>1.878694172783572</v>
+        <v>2.132809610101132</v>
       </c>
     </row>
     <row r="28">
@@ -1245,30 +1246,30 @@
         <v>2036</v>
       </c>
       <c r="B28" t="n">
-        <v>1.665774378432503</v>
+        <v>1.625483388423634</v>
       </c>
       <c r="C28" t="n">
-        <v>1.753442214466495</v>
+        <v>1.795645470142645</v>
       </c>
       <c r="D28" t="n">
-        <v>1.841110050500486</v>
+        <v>1.983620796993017</v>
       </c>
       <c r="E28" t="n">
-        <v>1.902810575210099</v>
+        <v>2.191274130494501</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>1.665774378432503</v>
+        <v>1.625483388423634</v>
       </c>
       <c r="I28" t="n">
-        <v>1.753442214466495</v>
+        <v>1.795645470142645</v>
       </c>
       <c r="J28" t="n">
-        <v>1.841110050500486</v>
+        <v>1.983620796993017</v>
       </c>
       <c r="K28" t="n">
-        <v>1.902810575210099</v>
+        <v>2.191274130494501</v>
       </c>
     </row>
     <row r="29">
@@ -1276,30 +1277,30 @@
         <v>2037</v>
       </c>
       <c r="B29" t="n">
-        <v>1.6894084516379</v>
+        <v>1.636145629531746</v>
       </c>
       <c r="C29" t="n">
-        <v>1.777076288111156</v>
+        <v>1.819279543787306</v>
       </c>
       <c r="D29" t="n">
-        <v>1.864744124584411</v>
+        <v>2.022911652057638</v>
       </c>
       <c r="E29" t="n">
-        <v>1.926444649603178</v>
+        <v>2.249336318876887</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>1.6894084516379</v>
+        <v>1.636145629531746</v>
       </c>
       <c r="I29" t="n">
-        <v>1.777076288111156</v>
+        <v>1.819279543787306</v>
       </c>
       <c r="J29" t="n">
-        <v>1.864744124584411</v>
+        <v>2.022911652057638</v>
       </c>
       <c r="K29" t="n">
-        <v>1.926444649603178</v>
+        <v>2.249336318876887</v>
       </c>
     </row>
     <row r="30">
@@ -1307,30 +1308,30 @@
         <v>2038</v>
       </c>
       <c r="B30" t="n">
-        <v>1.712569843370337</v>
+        <v>1.646527640378561</v>
       </c>
       <c r="C30" t="n">
-        <v>1.800237680282924</v>
+        <v>1.842440935959074</v>
       </c>
       <c r="D30" t="n">
-        <v>1.887905517195511</v>
+        <v>2.061665118307569</v>
       </c>
       <c r="E30" t="n">
-        <v>1.94960604252348</v>
+        <v>2.306973850335997</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>1.712569843370337</v>
+        <v>1.646527640378561</v>
       </c>
       <c r="I30" t="n">
-        <v>1.800237680282924</v>
+        <v>1.842440935959074</v>
       </c>
       <c r="J30" t="n">
-        <v>1.887905517195511</v>
+        <v>2.061665118307569</v>
       </c>
       <c r="K30" t="n">
-        <v>1.94960604252348</v>
+        <v>2.306973850335997</v>
       </c>
     </row>
     <row r="31">
@@ -1338,30 +1339,30 @@
         <v>2039</v>
       </c>
       <c r="B31" t="n">
-        <v>1.735268007259272</v>
+        <v>1.656638887940114</v>
       </c>
       <c r="C31" t="n">
-        <v>1.822935844611257</v>
+        <v>1.865139100287407</v>
       </c>
       <c r="D31" t="n">
-        <v>1.910603681963242</v>
+        <v>2.099880600863131</v>
       </c>
       <c r="E31" t="n">
-        <v>1.972304207600458</v>
+        <v>2.364166049171255</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>1.735268007259272</v>
+        <v>1.656638887940114</v>
       </c>
       <c r="I31" t="n">
-        <v>1.822935844611257</v>
+        <v>1.865139100287407</v>
       </c>
       <c r="J31" t="n">
-        <v>1.910603681963242</v>
+        <v>2.099880600863131</v>
       </c>
       <c r="K31" t="n">
-        <v>1.972304207600458</v>
+        <v>2.364166049171255</v>
       </c>
     </row>
     <row r="32">
@@ -1369,30 +1370,30 @@
         <v>2040</v>
       </c>
       <c r="B32" t="n">
-        <v>1.757512207861575</v>
+        <v>1.666488390853722</v>
       </c>
       <c r="C32" t="n">
-        <v>1.845180045653023</v>
+        <v>1.887383301329173</v>
       </c>
       <c r="D32" t="n">
-        <v>1.932847883444471</v>
+        <v>2.137558080624448</v>
       </c>
       <c r="E32" t="n">
-        <v>1.994548409390981</v>
+        <v>2.420893808282128</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>1.757512207861575</v>
+        <v>1.666488390853722</v>
       </c>
       <c r="I32" t="n">
-        <v>1.845180045653023</v>
+        <v>1.887383301329173</v>
       </c>
       <c r="J32" t="n">
-        <v>1.932847883444471</v>
+        <v>2.137558080624448</v>
       </c>
       <c r="K32" t="n">
-        <v>1.994548409390981</v>
+        <v>2.420893808282128</v>
       </c>
     </row>
     <row r="33">
@@ -1400,30 +1401,30 @@
         <v>2041</v>
       </c>
       <c r="B33" t="n">
-        <v>1.779311524442979</v>
+        <v>1.676084748939832</v>
       </c>
       <c r="C33" t="n">
-        <v>1.866979362673954</v>
+        <v>1.909182618350104</v>
       </c>
       <c r="D33" t="n">
-        <v>1.954647200904928</v>
+        <v>2.17469807091539</v>
       </c>
       <c r="E33" t="n">
-        <v>2.016347727160776</v>
+        <v>2.477139512054714</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>1.779311524442979</v>
+        <v>1.676084748939832</v>
       </c>
       <c r="I33" t="n">
-        <v>1.866979362673954</v>
+        <v>1.909182618350104</v>
       </c>
       <c r="J33" t="n">
-        <v>1.954647200904928</v>
+        <v>2.17469807091539</v>
       </c>
       <c r="K33" t="n">
-        <v>2.016347727160776</v>
+        <v>2.477139512054714</v>
       </c>
     </row>
     <row r="34">
@@ -1431,30 +1432,30 @@
         <v>2042</v>
       </c>
       <c r="B34" t="n">
-        <v>1.800674854683903</v>
+        <v>1.685436170203904</v>
       </c>
       <c r="C34" t="n">
-        <v>1.888342693354466</v>
+        <v>1.930545949030616</v>
       </c>
       <c r="D34" t="n">
-        <v>1.976010532025029</v>
+        <v>2.211301577126845</v>
       </c>
       <c r="E34" t="n">
-        <v>2.037711058590259</v>
+        <v>2.532886962601958</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>1.800674854683903</v>
+        <v>1.685436170203904</v>
       </c>
       <c r="I34" t="n">
-        <v>1.888342693354466</v>
+        <v>1.930545949030616</v>
       </c>
       <c r="J34" t="n">
-        <v>1.976010532025029</v>
+        <v>2.211301577126845</v>
       </c>
       <c r="K34" t="n">
-        <v>2.037711058590259</v>
+        <v>2.532886962601958</v>
       </c>
     </row>
     <row r="35">
@@ -1462,30 +1463,30 @@
         <v>2043</v>
       </c>
       <c r="B35" t="n">
-        <v>1.821610918311155</v>
+        <v>1.694550495580007</v>
       </c>
       <c r="C35" t="n">
-        <v>1.909278757421368</v>
+        <v>1.951482013097518</v>
       </c>
       <c r="D35" t="n">
-        <v>1.996946596531581</v>
+        <v>2.247370059125709</v>
       </c>
       <c r="E35" t="n">
-        <v>2.058647123406236</v>
+        <v>2.588121309218701</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>1.821610918311155</v>
+        <v>1.694550495580007</v>
       </c>
       <c r="I35" t="n">
-        <v>1.909278757421368</v>
+        <v>1.951482013097518</v>
       </c>
       <c r="J35" t="n">
-        <v>1.996946596531581</v>
+        <v>2.247370059125709</v>
       </c>
       <c r="K35" t="n">
-        <v>2.058647123406236</v>
+        <v>2.588121309218701</v>
       </c>
     </row>
     <row r="36">
@@ -1493,30 +1494,30 @@
         <v>2044</v>
       </c>
       <c r="B36" t="n">
-        <v>1.842128260657009</v>
+        <v>1.703435221646106</v>
       </c>
       <c r="C36" t="n">
-        <v>1.929796100206932</v>
+        <v>1.971999355883082</v>
       </c>
       <c r="D36" t="n">
-        <v>2.017463939756855</v>
+        <v>2.282905396217759</v>
       </c>
       <c r="E36" t="n">
-        <v>2.079164466940977</v>
+        <v>2.642828980918369</v>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>1.842128260657009</v>
+        <v>1.703435221646106</v>
       </c>
       <c r="I36" t="n">
-        <v>1.929796100206932</v>
+        <v>1.971999355883082</v>
       </c>
       <c r="J36" t="n">
-        <v>2.017463939756855</v>
+        <v>2.282905396217759</v>
       </c>
       <c r="K36" t="n">
-        <v>2.079164466940977</v>
+        <v>2.642828980918369</v>
       </c>
     </row>
     <row r="37">
@@ -1524,30 +1525,30 @@
         <v>2045</v>
       </c>
       <c r="B37" t="n">
-        <v>1.862235256147094</v>
+        <v>1.712097521513627</v>
       </c>
       <c r="C37" t="n">
-        <v>1.949903096136785</v>
+        <v>1.992106351812934</v>
       </c>
       <c r="D37" t="n">
-        <v>2.037570936126476</v>
+        <v>2.317909854471951</v>
       </c>
       <c r="E37" t="n">
-        <v>2.099271463620106</v>
+        <v>2.696997621923499</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>1.862235256147094</v>
+        <v>1.712097521513627</v>
       </c>
       <c r="I37" t="n">
-        <v>1.949903096136785</v>
+        <v>1.992106351812934</v>
       </c>
       <c r="J37" t="n">
-        <v>2.037570936126476</v>
+        <v>2.317909854471951</v>
       </c>
       <c r="K37" t="n">
-        <v>2.099271463620106</v>
+        <v>2.696997621923499</v>
       </c>
     </row>
     <row r="38">
@@ -1555,30 +1556,30 @@
         <v>2046</v>
       </c>
       <c r="B38" t="n">
-        <v>1.881940111718524</v>
+        <v>1.720544264070273</v>
       </c>
       <c r="C38" t="n">
-        <v>1.969607952148041</v>
+        <v>2.01181120782419</v>
       </c>
       <c r="D38" t="n">
-        <v>2.057275792577557</v>
+        <v>2.352386056230934</v>
       </c>
       <c r="E38" t="n">
-        <v>2.118976320380736</v>
+        <v>2.750616029987499</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>1.881940111718524</v>
+        <v>1.720544264070273</v>
       </c>
       <c r="I38" t="n">
-        <v>1.969607952148041</v>
+        <v>2.01181120782419</v>
       </c>
       <c r="J38" t="n">
-        <v>2.057275792577557</v>
+        <v>2.352386056230934</v>
       </c>
       <c r="K38" t="n">
-        <v>2.118976320380736</v>
+        <v>2.750616029987499</v>
       </c>
     </row>
     <row r="39">
@@ -1586,30 +1587,30 @@
         <v>2047</v>
       </c>
       <c r="B39" t="n">
-        <v>1.901250870169673</v>
+        <v>1.728782031734508</v>
       </c>
       <c r="C39" t="n">
-        <v>1.988918711039071</v>
+        <v>2.03112196671522</v>
       </c>
       <c r="D39" t="n">
-        <v>2.076586551908469</v>
+        <v>2.386336951647967</v>
       </c>
       <c r="E39" t="n">
-        <v>2.138287080021236</v>
+        <v>2.803674097429985</v>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>1.901250870169673</v>
+        <v>1.728782031734508</v>
       </c>
       <c r="I39" t="n">
-        <v>1.988918711039071</v>
+        <v>2.03112196671522</v>
       </c>
       <c r="J39" t="n">
-        <v>2.076586551908469</v>
+        <v>2.386336951647967</v>
       </c>
       <c r="K39" t="n">
-        <v>2.138287080021236</v>
+        <v>2.803674097429985</v>
       </c>
     </row>
     <row r="40">
@@ -1617,30 +1618,30 @@
         <v>2048</v>
       </c>
       <c r="B40" t="n">
-        <v>1.920175413442945</v>
+        <v>1.736817136862315</v>
       </c>
       <c r="C40" t="n">
-        <v>2.007843254752281</v>
+        <v>2.050046510428431</v>
       </c>
       <c r="D40" t="n">
-        <v>2.095511096061616</v>
+        <v>2.419765792104198</v>
       </c>
       <c r="E40" t="n">
-        <v>2.15721162448401</v>
+        <v>2.856162754772812</v>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>1.920175413442945</v>
+        <v>1.736817136862315</v>
       </c>
       <c r="I40" t="n">
-        <v>2.007843254752281</v>
+        <v>2.050046510428431</v>
       </c>
       <c r="J40" t="n">
-        <v>2.095511096061616</v>
+        <v>2.419765792104198</v>
       </c>
       <c r="K40" t="n">
-        <v>2.15721162448401</v>
+        <v>2.856162754772812</v>
       </c>
     </row>
     <row r="41">
@@ -1648,30 +1649,30 @@
         <v>2049</v>
       </c>
       <c r="B41" t="n">
-        <v>1.9387214658419</v>
+        <v>1.744655636931287</v>
       </c>
       <c r="C41" t="n">
-        <v>2.026389307591226</v>
+        <v>2.068592563267376</v>
       </c>
       <c r="D41" t="n">
-        <v>2.114057149340553</v>
+        <v>2.452676105372664</v>
       </c>
       <c r="E41" t="n">
-        <v>2.175757678072613</v>
+        <v>2.908073916868505</v>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>1.9387214658419</v>
+        <v>1.744655636931287</v>
       </c>
       <c r="I41" t="n">
-        <v>2.026389307591226</v>
+        <v>2.068592563267376</v>
       </c>
       <c r="J41" t="n">
-        <v>2.114057149340553</v>
+        <v>2.452676105372664</v>
       </c>
       <c r="K41" t="n">
-        <v>2.175757678072613</v>
+        <v>2.908073916868505</v>
       </c>
     </row>
     <row r="42">
@@ -1679,30 +1680,30 @@
         <v>2050</v>
       </c>
       <c r="B42" t="n">
-        <v>1.956896597184022</v>
+        <v>1.752303348613496</v>
       </c>
       <c r="C42" t="n">
-        <v>2.044564439373393</v>
+        <v>2.086767695049543</v>
       </c>
       <c r="D42" t="n">
-        <v>2.132232281562764</v>
+        <v>2.485071672406462</v>
       </c>
       <c r="E42" t="n">
-        <v>2.193932810604526</v>
+        <v>2.959400431417178</v>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>1.956896597184022</v>
+        <v>1.752303348613496</v>
       </c>
       <c r="I42" t="n">
-        <v>2.044564439373393</v>
+        <v>2.086767695049543</v>
       </c>
       <c r="J42" t="n">
-        <v>2.132232281562764</v>
+        <v>2.485071672406462</v>
       </c>
       <c r="K42" t="n">
-        <v>2.193932810604526</v>
+        <v>2.959400431417178</v>
       </c>
     </row>
   </sheetData>
@@ -1796,7 +1797,7 @@
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9369887862582014</v>
+        <v>0.9791920419343512</v>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
@@ -1823,7 +1824,7 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9769583215142472</v>
+        <v>1.019161577190397</v>
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
@@ -1850,7 +1851,7 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>1.016124595359883</v>
+        <v>1.058327851036033</v>
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
@@ -1877,7 +1878,7 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>1.054503673026557</v>
+        <v>1.096706928702707</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
@@ -1904,7 +1905,7 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>1.092111298448804</v>
+        <v>1.134314554124954</v>
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
@@ -1931,7 +1932,7 @@
         <v>1.153908543682574</v>
       </c>
       <c r="G7" t="n">
-        <v>1.128962900690027</v>
+        <v>1.171166156366177</v>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
@@ -1958,7 +1959,7 @@
         <v>1.14257096572451</v>
       </c>
       <c r="G8" t="n">
-        <v>1.165088992602441</v>
+        <v>1.207292248278591</v>
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
@@ -1985,7 +1986,7 @@
         <v>1.208048138561229</v>
       </c>
       <c r="G9" t="n">
-        <v>1.200487865980228</v>
+        <v>1.242691121656378</v>
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
@@ -2012,7 +2013,7 @@
         <v>1.215777713114327</v>
       </c>
       <c r="G10" t="n">
-        <v>1.235181724758443</v>
+        <v>1.277384980434593</v>
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
@@ -2039,7 +2040,7 @@
         <v>1.358509372339871</v>
       </c>
       <c r="G11" t="n">
-        <v>1.269179024863056</v>
+        <v>1.311382280539206</v>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
@@ -2066,7 +2067,7 @@
         <v>1.105484425759602</v>
       </c>
       <c r="G12" t="n">
-        <v>1.302507214468904</v>
+        <v>1.344710470145054</v>
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
@@ -2093,7 +2094,7 @@
         <v>1.276148524225631</v>
       </c>
       <c r="G13" t="n">
-        <v>1.335140381698887</v>
+        <v>1.377343637375037</v>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
@@ -2120,7 +2121,7 @@
         <v>1.49238768827198</v>
       </c>
       <c r="G14" t="n">
-        <v>1.367134294053697</v>
+        <v>1.409337549729847</v>
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
@@ -2147,7 +2148,7 @@
         <v>1.438405529593662</v>
       </c>
       <c r="G15" t="n">
-        <v>1.398506635930348</v>
+        <v>1.440709891606498</v>
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
@@ -2174,19 +2175,19 @@
         <v>1.471446502093358</v>
       </c>
       <c r="G16" t="n">
-        <v>1.429243246417209</v>
+        <v>1.471446502093358</v>
       </c>
       <c r="H16" t="n">
-        <v>1.341575415210259</v>
+        <v>1.471446502093358</v>
       </c>
       <c r="I16" t="n">
-        <v>1.429243246417209</v>
+        <v>1.471446502093358</v>
       </c>
       <c r="J16" t="n">
-        <v>1.516911077624158</v>
+        <v>1.471446502093358</v>
       </c>
       <c r="K16" t="n">
-        <v>1.578611598936505</v>
+        <v>1.471446502093358</v>
       </c>
     </row>
     <row r="17">
@@ -2194,30 +2195,30 @@
         <v>2025</v>
       </c>
       <c r="B17" t="n">
-        <v>1.371697604134962</v>
+        <v>1.486431296108713</v>
       </c>
       <c r="C17" t="n">
-        <v>1.459365435341912</v>
+        <v>1.501568691018062</v>
       </c>
       <c r="D17" t="n">
-        <v>1.547033266548862</v>
+        <v>1.516860240865645</v>
       </c>
       <c r="E17" t="n">
-        <v>1.608733787861209</v>
+        <v>1.532307515521649</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>1.371697604134962</v>
+        <v>1.486431296108713</v>
       </c>
       <c r="I17" t="n">
-        <v>1.459365435341912</v>
+        <v>1.501568691018062</v>
       </c>
       <c r="J17" t="n">
-        <v>1.547033266548862</v>
+        <v>1.516860240865645</v>
       </c>
       <c r="K17" t="n">
-        <v>1.608733787861209</v>
+        <v>1.532307515521649</v>
       </c>
     </row>
     <row r="18">
@@ -2225,30 +2226,30 @@
         <v>2026</v>
       </c>
       <c r="B18" t="n">
-        <v>1.40121321292369</v>
+        <v>1.500969232864511</v>
       </c>
       <c r="C18" t="n">
-        <v>1.488881044569065</v>
+        <v>1.531084300245215</v>
       </c>
       <c r="D18" t="n">
-        <v>1.57654887621444</v>
+        <v>1.561803588727516</v>
       </c>
       <c r="E18" t="n">
-        <v>1.63824939783535</v>
+        <v>1.593139221250904</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>1.40121321292369</v>
+        <v>1.500969232864511</v>
       </c>
       <c r="I18" t="n">
-        <v>1.488881044569065</v>
+        <v>1.531084300245215</v>
       </c>
       <c r="J18" t="n">
-        <v>1.57654887621444</v>
+        <v>1.561803588727516</v>
       </c>
       <c r="K18" t="n">
-        <v>1.63824939783535</v>
+        <v>1.593139221250904</v>
       </c>
     </row>
     <row r="19">
@@ -2256,30 +2257,30 @@
         <v>2027</v>
       </c>
       <c r="B19" t="n">
-        <v>1.430138509527791</v>
+        <v>1.515081075441588</v>
       </c>
       <c r="C19" t="n">
-        <v>1.517806341611675</v>
+        <v>1.560009597287825</v>
       </c>
       <c r="D19" t="n">
-        <v>1.605474173695559</v>
+        <v>1.606270438643564</v>
       </c>
       <c r="E19" t="n">
-        <v>1.667174695625092</v>
+        <v>1.653903108382065</v>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>1.430138509527791</v>
+        <v>1.515081075441588</v>
       </c>
       <c r="I19" t="n">
-        <v>1.517806341611675</v>
+        <v>1.560009597287825</v>
       </c>
       <c r="J19" t="n">
-        <v>1.605474173695559</v>
+        <v>1.606270438643564</v>
       </c>
       <c r="K19" t="n">
-        <v>1.667174695625092</v>
+        <v>1.653903108382065</v>
       </c>
     </row>
     <row r="20">
@@ -2287,30 +2288,30 @@
         <v>2028</v>
       </c>
       <c r="B20" t="n">
-        <v>1.458485300190957</v>
+        <v>1.528784305182877</v>
       </c>
       <c r="C20" t="n">
-        <v>1.546153132713433</v>
+        <v>1.588356388389583</v>
       </c>
       <c r="D20" t="n">
-        <v>1.633820965235909</v>
+        <v>1.650249814826694</v>
       </c>
       <c r="E20" t="n">
-        <v>1.695521487474122</v>
+        <v>1.714555040192641</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>1.458485300190957</v>
+        <v>1.528784305182877</v>
       </c>
       <c r="I20" t="n">
-        <v>1.546153132713433</v>
+        <v>1.588356388389583</v>
       </c>
       <c r="J20" t="n">
-        <v>1.633820965235909</v>
+        <v>1.650249814826694</v>
       </c>
       <c r="K20" t="n">
-        <v>1.695521487474122</v>
+        <v>1.714555040192641</v>
       </c>
     </row>
     <row r="21">
@@ -2318,30 +2319,30 @@
         <v>2029</v>
       </c>
       <c r="B21" t="n">
-        <v>1.486265155032007</v>
+        <v>1.542095335137714</v>
       </c>
       <c r="C21" t="n">
-        <v>1.573932987993156</v>
+        <v>1.616136243669305</v>
       </c>
       <c r="D21" t="n">
-        <v>1.661600820954304</v>
+        <v>1.693732092035854</v>
       </c>
       <c r="E21" t="n">
-        <v>1.723301343501254</v>
+        <v>1.775053564221132</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>1.486265155032007</v>
+        <v>1.542095335137714</v>
       </c>
       <c r="I21" t="n">
-        <v>1.573932987993156</v>
+        <v>1.616136243669305</v>
       </c>
       <c r="J21" t="n">
-        <v>1.661600820954304</v>
+        <v>1.693732092035854</v>
       </c>
       <c r="K21" t="n">
-        <v>1.723301343501254</v>
+        <v>1.775053564221132</v>
       </c>
     </row>
     <row r="22">
@@ -2349,30 +2350,30 @@
         <v>2030</v>
       </c>
       <c r="B22" t="n">
-        <v>1.513489412767383</v>
+        <v>1.555029601684774</v>
       </c>
       <c r="C22" t="n">
-        <v>1.601157246167284</v>
+        <v>1.643360501843434</v>
       </c>
       <c r="D22" t="n">
-        <v>1.688825079567184</v>
+        <v>1.736708893575492</v>
       </c>
       <c r="E22" t="n">
-        <v>1.750525602422928</v>
+        <v>1.835359787241355</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>1.513489412767383</v>
+        <v>1.555029601684774</v>
       </c>
       <c r="I22" t="n">
-        <v>1.601157246167284</v>
+        <v>1.643360501843434</v>
       </c>
       <c r="J22" t="n">
-        <v>1.688825079567184</v>
+        <v>1.736708893575492</v>
       </c>
       <c r="K22" t="n">
-        <v>1.750525602422928</v>
+        <v>1.835359787241355</v>
       </c>
     </row>
     <row r="23">
@@ -2380,30 +2381,30 @@
         <v>2031</v>
       </c>
       <c r="B23" t="n">
-        <v>1.540169185339199</v>
+        <v>1.567601646078833</v>
       </c>
       <c r="C23" t="n">
-        <v>1.627837019177929</v>
+        <v>1.670040274854079</v>
       </c>
       <c r="D23" t="n">
-        <v>1.71550485301666</v>
+        <v>1.779172997560397</v>
       </c>
       <c r="E23" t="n">
-        <v>1.777205376181251</v>
+        <v>1.895437255562373</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>1.540169185339199</v>
+        <v>1.567601646078833</v>
       </c>
       <c r="I23" t="n">
-        <v>1.627837019177929</v>
+        <v>1.670040274854079</v>
       </c>
       <c r="J23" t="n">
-        <v>1.71550485301666</v>
+        <v>1.779172997560397</v>
       </c>
       <c r="K23" t="n">
-        <v>1.777205376181251</v>
+        <v>1.895437255562373</v>
       </c>
     </row>
     <row r="24">
@@ -2411,30 +2412,30 @@
         <v>2032</v>
       </c>
       <c r="B24" t="n">
-        <v>1.566315362450726</v>
+        <v>1.579825187256097</v>
       </c>
       <c r="C24" t="n">
-        <v>1.653983196728362</v>
+        <v>1.696186452404512</v>
       </c>
       <c r="D24" t="n">
-        <v>1.741651031005998</v>
+        <v>1.821118250632258</v>
       </c>
       <c r="E24" t="n">
-        <v>1.803351554479491</v>
+        <v>1.955251840435626</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>1.566315362450726</v>
+        <v>1.579825187256097</v>
       </c>
       <c r="I24" t="n">
-        <v>1.653983196728362</v>
+        <v>1.696186452404512</v>
       </c>
       <c r="J24" t="n">
-        <v>1.741651031005998</v>
+        <v>1.821118250632258</v>
       </c>
       <c r="K24" t="n">
-        <v>1.803351554479491</v>
+        <v>1.955251840435626</v>
       </c>
     </row>
     <row r="25">
@@ -2442,30 +2443,30 @@
         <v>2033</v>
       </c>
       <c r="B25" t="n">
-        <v>1.59193861601117</v>
+        <v>1.591713187027884</v>
       </c>
       <c r="C25" t="n">
-        <v>1.679606450727786</v>
+        <v>1.721809706403936</v>
       </c>
       <c r="D25" t="n">
-        <v>1.767274285444403</v>
+        <v>1.862539488412791</v>
       </c>
       <c r="E25" t="n">
-        <v>1.828974809226849</v>
+        <v>2.014771628359691</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>1.59193861601117</v>
+        <v>1.591713187027884</v>
       </c>
       <c r="I25" t="n">
-        <v>1.679606450727786</v>
+        <v>1.721809706403936</v>
       </c>
       <c r="J25" t="n">
-        <v>1.767274285444403</v>
+        <v>1.862539488412791</v>
       </c>
       <c r="K25" t="n">
-        <v>1.828974809226849</v>
+        <v>2.014771628359691</v>
       </c>
     </row>
     <row r="26">
@@ -2473,30 +2474,30 @@
         <v>2034</v>
       </c>
       <c r="B26" t="n">
-        <v>1.617049404491552</v>
+        <v>1.603277908623072</v>
       </c>
       <c r="C26" t="n">
-        <v>1.704717239647222</v>
+        <v>1.746920495323371</v>
       </c>
       <c r="D26" t="n">
-        <v>1.792385074802892</v>
+        <v>1.903432462062515</v>
       </c>
       <c r="E26" t="n">
-        <v>1.854085598894344</v>
+        <v>2.073966816081521</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>1.617049404491552</v>
+        <v>1.603277908623072</v>
       </c>
       <c r="I26" t="n">
-        <v>1.704717239647222</v>
+        <v>1.746920495323371</v>
       </c>
       <c r="J26" t="n">
-        <v>1.792385074802892</v>
+        <v>1.903432462062515</v>
       </c>
       <c r="K26" t="n">
-        <v>1.854085598894344</v>
+        <v>2.073966816081521</v>
       </c>
     </row>
     <row r="27">
@@ -2504,30 +2505,30 @@
         <v>2035</v>
       </c>
       <c r="B27" t="n">
-        <v>1.641657977193473</v>
+        <v>1.614530969399062</v>
       </c>
       <c r="C27" t="n">
-        <v>1.729325812788269</v>
+        <v>1.771529068464418</v>
       </c>
       <c r="D27" t="n">
-        <v>1.816993648383064</v>
+        <v>1.94379377038677</v>
       </c>
       <c r="E27" t="n">
-        <v>1.878694172783572</v>
+        <v>2.132809610101132</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>1.641657977193473</v>
+        <v>1.614530969399062</v>
       </c>
       <c r="I27" t="n">
-        <v>1.729325812788269</v>
+        <v>1.771529068464418</v>
       </c>
       <c r="J27" t="n">
-        <v>1.816993648383064</v>
+        <v>1.94379377038677</v>
       </c>
       <c r="K27" t="n">
-        <v>1.878694172783572</v>
+        <v>2.132809610101132</v>
       </c>
     </row>
     <row r="28">
@@ -2535,30 +2536,30 @@
         <v>2036</v>
       </c>
       <c r="B28" t="n">
-        <v>1.665774378432503</v>
+        <v>1.625483388423634</v>
       </c>
       <c r="C28" t="n">
-        <v>1.753442214466495</v>
+        <v>1.795645470142645</v>
       </c>
       <c r="D28" t="n">
-        <v>1.841110050500486</v>
+        <v>1.983620796993017</v>
       </c>
       <c r="E28" t="n">
-        <v>1.902810575210099</v>
+        <v>2.191274130494501</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>1.665774378432503</v>
+        <v>1.625483388423634</v>
       </c>
       <c r="I28" t="n">
-        <v>1.753442214466495</v>
+        <v>1.795645470142645</v>
       </c>
       <c r="J28" t="n">
-        <v>1.841110050500486</v>
+        <v>1.983620796993017</v>
       </c>
       <c r="K28" t="n">
-        <v>1.902810575210099</v>
+        <v>2.191274130494501</v>
       </c>
     </row>
     <row r="29">
@@ -2566,30 +2567,30 @@
         <v>2037</v>
       </c>
       <c r="B29" t="n">
-        <v>1.6894084516379</v>
+        <v>1.636145629531746</v>
       </c>
       <c r="C29" t="n">
-        <v>1.777076288111156</v>
+        <v>1.819279543787306</v>
       </c>
       <c r="D29" t="n">
-        <v>1.864744124584411</v>
+        <v>2.022911652057638</v>
       </c>
       <c r="E29" t="n">
-        <v>1.926444649603178</v>
+        <v>2.249336318876887</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>1.6894084516379</v>
+        <v>1.636145629531746</v>
       </c>
       <c r="I29" t="n">
-        <v>1.777076288111156</v>
+        <v>1.819279543787306</v>
       </c>
       <c r="J29" t="n">
-        <v>1.864744124584411</v>
+        <v>2.022911652057638</v>
       </c>
       <c r="K29" t="n">
-        <v>1.926444649603178</v>
+        <v>2.249336318876887</v>
       </c>
     </row>
     <row r="30">
@@ -2597,30 +2598,30 @@
         <v>2038</v>
       </c>
       <c r="B30" t="n">
-        <v>1.712569843370337</v>
+        <v>1.646527640378561</v>
       </c>
       <c r="C30" t="n">
-        <v>1.800237680282924</v>
+        <v>1.842440935959074</v>
       </c>
       <c r="D30" t="n">
-        <v>1.887905517195511</v>
+        <v>2.061665118307569</v>
       </c>
       <c r="E30" t="n">
-        <v>1.94960604252348</v>
+        <v>2.306973850335997</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>1.712569843370337</v>
+        <v>1.646527640378561</v>
       </c>
       <c r="I30" t="n">
-        <v>1.800237680282924</v>
+        <v>1.842440935959074</v>
       </c>
       <c r="J30" t="n">
-        <v>1.887905517195511</v>
+        <v>2.061665118307569</v>
       </c>
       <c r="K30" t="n">
-        <v>1.94960604252348</v>
+        <v>2.306973850335997</v>
       </c>
     </row>
     <row r="31">
@@ -2628,30 +2629,30 @@
         <v>2039</v>
       </c>
       <c r="B31" t="n">
-        <v>1.735268007259272</v>
+        <v>1.656638887940114</v>
       </c>
       <c r="C31" t="n">
-        <v>1.822935844611257</v>
+        <v>1.865139100287407</v>
       </c>
       <c r="D31" t="n">
-        <v>1.910603681963242</v>
+        <v>2.099880600863131</v>
       </c>
       <c r="E31" t="n">
-        <v>1.972304207600458</v>
+        <v>2.364166049171255</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>1.735268007259272</v>
+        <v>1.656638887940114</v>
       </c>
       <c r="I31" t="n">
-        <v>1.822935844611257</v>
+        <v>1.865139100287407</v>
       </c>
       <c r="J31" t="n">
-        <v>1.910603681963242</v>
+        <v>2.099880600863131</v>
       </c>
       <c r="K31" t="n">
-        <v>1.972304207600458</v>
+        <v>2.364166049171255</v>
       </c>
     </row>
     <row r="32">
@@ -2659,30 +2660,30 @@
         <v>2040</v>
       </c>
       <c r="B32" t="n">
-        <v>1.757512207861575</v>
+        <v>1.666488390853722</v>
       </c>
       <c r="C32" t="n">
-        <v>1.845180045653023</v>
+        <v>1.887383301329173</v>
       </c>
       <c r="D32" t="n">
-        <v>1.932847883444471</v>
+        <v>2.137558080624448</v>
       </c>
       <c r="E32" t="n">
-        <v>1.994548409390981</v>
+        <v>2.420893808282128</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>1.757512207861575</v>
+        <v>1.666488390853722</v>
       </c>
       <c r="I32" t="n">
-        <v>1.845180045653023</v>
+        <v>1.887383301329173</v>
       </c>
       <c r="J32" t="n">
-        <v>1.932847883444471</v>
+        <v>2.137558080624448</v>
       </c>
       <c r="K32" t="n">
-        <v>1.994548409390981</v>
+        <v>2.420893808282128</v>
       </c>
     </row>
     <row r="33">
@@ -2690,30 +2691,30 @@
         <v>2041</v>
       </c>
       <c r="B33" t="n">
-        <v>1.779311524442979</v>
+        <v>1.676084748939832</v>
       </c>
       <c r="C33" t="n">
-        <v>1.866979362673954</v>
+        <v>1.909182618350104</v>
       </c>
       <c r="D33" t="n">
-        <v>1.954647200904928</v>
+        <v>2.17469807091539</v>
       </c>
       <c r="E33" t="n">
-        <v>2.016347727160776</v>
+        <v>2.477139512054714</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>1.779311524442979</v>
+        <v>1.676084748939832</v>
       </c>
       <c r="I33" t="n">
-        <v>1.866979362673954</v>
+        <v>1.909182618350104</v>
       </c>
       <c r="J33" t="n">
-        <v>1.954647200904928</v>
+        <v>2.17469807091539</v>
       </c>
       <c r="K33" t="n">
-        <v>2.016347727160776</v>
+        <v>2.477139512054714</v>
       </c>
     </row>
     <row r="34">
@@ -2721,30 +2722,30 @@
         <v>2042</v>
       </c>
       <c r="B34" t="n">
-        <v>1.800674854683903</v>
+        <v>1.685436170203904</v>
       </c>
       <c r="C34" t="n">
-        <v>1.888342693354466</v>
+        <v>1.930545949030616</v>
       </c>
       <c r="D34" t="n">
-        <v>1.976010532025029</v>
+        <v>2.211301577126845</v>
       </c>
       <c r="E34" t="n">
-        <v>2.037711058590259</v>
+        <v>2.532886962601958</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>1.800674854683903</v>
+        <v>1.685436170203904</v>
       </c>
       <c r="I34" t="n">
-        <v>1.888342693354466</v>
+        <v>1.930545949030616</v>
       </c>
       <c r="J34" t="n">
-        <v>1.976010532025029</v>
+        <v>2.211301577126845</v>
       </c>
       <c r="K34" t="n">
-        <v>2.037711058590259</v>
+        <v>2.532886962601958</v>
       </c>
     </row>
     <row r="35">
@@ -2752,30 +2753,30 @@
         <v>2043</v>
       </c>
       <c r="B35" t="n">
-        <v>1.821610918311155</v>
+        <v>1.694550495580007</v>
       </c>
       <c r="C35" t="n">
-        <v>1.909278757421368</v>
+        <v>1.951482013097518</v>
       </c>
       <c r="D35" t="n">
-        <v>1.996946596531581</v>
+        <v>2.247370059125709</v>
       </c>
       <c r="E35" t="n">
-        <v>2.058647123406236</v>
+        <v>2.588121309218701</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>1.821610918311155</v>
+        <v>1.694550495580007</v>
       </c>
       <c r="I35" t="n">
-        <v>1.909278757421368</v>
+        <v>1.951482013097518</v>
       </c>
       <c r="J35" t="n">
-        <v>1.996946596531581</v>
+        <v>2.247370059125709</v>
       </c>
       <c r="K35" t="n">
-        <v>2.058647123406236</v>
+        <v>2.588121309218701</v>
       </c>
     </row>
     <row r="36">
@@ -2783,30 +2784,30 @@
         <v>2044</v>
       </c>
       <c r="B36" t="n">
-        <v>1.842128260657009</v>
+        <v>1.703435221646106</v>
       </c>
       <c r="C36" t="n">
-        <v>1.929796100206932</v>
+        <v>1.971999355883082</v>
       </c>
       <c r="D36" t="n">
-        <v>2.017463939756855</v>
+        <v>2.282905396217759</v>
       </c>
       <c r="E36" t="n">
-        <v>2.079164466940977</v>
+        <v>2.642828980918369</v>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>1.842128260657009</v>
+        <v>1.703435221646106</v>
       </c>
       <c r="I36" t="n">
-        <v>1.929796100206932</v>
+        <v>1.971999355883082</v>
       </c>
       <c r="J36" t="n">
-        <v>2.017463939756855</v>
+        <v>2.282905396217759</v>
       </c>
       <c r="K36" t="n">
-        <v>2.079164466940977</v>
+        <v>2.642828980918369</v>
       </c>
     </row>
     <row r="37">
@@ -2814,30 +2815,30 @@
         <v>2045</v>
       </c>
       <c r="B37" t="n">
-        <v>1.862235256147094</v>
+        <v>1.712097521513627</v>
       </c>
       <c r="C37" t="n">
-        <v>1.949903096136785</v>
+        <v>1.992106351812934</v>
       </c>
       <c r="D37" t="n">
-        <v>2.037570936126476</v>
+        <v>2.317909854471951</v>
       </c>
       <c r="E37" t="n">
-        <v>2.099271463620106</v>
+        <v>2.696997621923499</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>1.862235256147094</v>
+        <v>1.712097521513627</v>
       </c>
       <c r="I37" t="n">
-        <v>1.949903096136785</v>
+        <v>1.992106351812934</v>
       </c>
       <c r="J37" t="n">
-        <v>2.037570936126476</v>
+        <v>2.317909854471951</v>
       </c>
       <c r="K37" t="n">
-        <v>2.099271463620106</v>
+        <v>2.696997621923499</v>
       </c>
     </row>
     <row r="38">
@@ -2845,30 +2846,30 @@
         <v>2046</v>
       </c>
       <c r="B38" t="n">
-        <v>1.881940111718524</v>
+        <v>1.720544264070273</v>
       </c>
       <c r="C38" t="n">
-        <v>1.969607952148041</v>
+        <v>2.01181120782419</v>
       </c>
       <c r="D38" t="n">
-        <v>2.057275792577557</v>
+        <v>2.352386056230934</v>
       </c>
       <c r="E38" t="n">
-        <v>2.118976320380736</v>
+        <v>2.750616029987499</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>1.881940111718524</v>
+        <v>1.720544264070273</v>
       </c>
       <c r="I38" t="n">
-        <v>1.969607952148041</v>
+        <v>2.01181120782419</v>
       </c>
       <c r="J38" t="n">
-        <v>2.057275792577557</v>
+        <v>2.352386056230934</v>
       </c>
       <c r="K38" t="n">
-        <v>2.118976320380736</v>
+        <v>2.750616029987499</v>
       </c>
     </row>
     <row r="39">
@@ -2876,30 +2877,30 @@
         <v>2047</v>
       </c>
       <c r="B39" t="n">
-        <v>1.901250870169673</v>
+        <v>1.728782031734508</v>
       </c>
       <c r="C39" t="n">
-        <v>1.988918711039071</v>
+        <v>2.03112196671522</v>
       </c>
       <c r="D39" t="n">
-        <v>2.076586551908469</v>
+        <v>2.386336951647967</v>
       </c>
       <c r="E39" t="n">
-        <v>2.138287080021236</v>
+        <v>2.803674097429985</v>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>1.901250870169673</v>
+        <v>1.728782031734508</v>
       </c>
       <c r="I39" t="n">
-        <v>1.988918711039071</v>
+        <v>2.03112196671522</v>
       </c>
       <c r="J39" t="n">
-        <v>2.076586551908469</v>
+        <v>2.386336951647967</v>
       </c>
       <c r="K39" t="n">
-        <v>2.138287080021236</v>
+        <v>2.803674097429985</v>
       </c>
     </row>
     <row r="40">
@@ -2907,30 +2908,30 @@
         <v>2048</v>
       </c>
       <c r="B40" t="n">
-        <v>1.920175413442945</v>
+        <v>1.736817136862315</v>
       </c>
       <c r="C40" t="n">
-        <v>2.007843254752281</v>
+        <v>2.050046510428431</v>
       </c>
       <c r="D40" t="n">
-        <v>2.095511096061616</v>
+        <v>2.419765792104198</v>
       </c>
       <c r="E40" t="n">
-        <v>2.15721162448401</v>
+        <v>2.856162754772812</v>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>1.920175413442945</v>
+        <v>1.736817136862315</v>
       </c>
       <c r="I40" t="n">
-        <v>2.007843254752281</v>
+        <v>2.050046510428431</v>
       </c>
       <c r="J40" t="n">
-        <v>2.095511096061616</v>
+        <v>2.419765792104198</v>
       </c>
       <c r="K40" t="n">
-        <v>2.15721162448401</v>
+        <v>2.856162754772812</v>
       </c>
     </row>
     <row r="41">
@@ -2938,30 +2939,30 @@
         <v>2049</v>
       </c>
       <c r="B41" t="n">
-        <v>1.9387214658419</v>
+        <v>1.744655636931287</v>
       </c>
       <c r="C41" t="n">
-        <v>2.026389307591226</v>
+        <v>2.068592563267376</v>
       </c>
       <c r="D41" t="n">
-        <v>2.114057149340553</v>
+        <v>2.452676105372664</v>
       </c>
       <c r="E41" t="n">
-        <v>2.175757678072613</v>
+        <v>2.908073916868505</v>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>1.9387214658419</v>
+        <v>1.744655636931287</v>
       </c>
       <c r="I41" t="n">
-        <v>2.026389307591226</v>
+        <v>2.068592563267376</v>
       </c>
       <c r="J41" t="n">
-        <v>2.114057149340553</v>
+        <v>2.452676105372664</v>
       </c>
       <c r="K41" t="n">
-        <v>2.175757678072613</v>
+        <v>2.908073916868505</v>
       </c>
     </row>
     <row r="42">
@@ -2969,30 +2970,164 @@
         <v>2050</v>
       </c>
       <c r="B42" t="n">
-        <v>1.956896597184022</v>
+        <v>1.752303348613496</v>
       </c>
       <c r="C42" t="n">
-        <v>2.044564439373393</v>
+        <v>2.086767695049543</v>
       </c>
       <c r="D42" t="n">
-        <v>2.132232281562764</v>
+        <v>2.485071672406462</v>
       </c>
       <c r="E42" t="n">
-        <v>2.193932810604526</v>
+        <v>2.959400431417178</v>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>1.956896597184022</v>
+        <v>1.752303348613496</v>
       </c>
       <c r="I42" t="n">
-        <v>2.044564439373393</v>
+        <v>2.086767695049543</v>
       </c>
       <c r="J42" t="n">
-        <v>2.132232281562764</v>
+        <v>2.485071672406462</v>
       </c>
       <c r="K42" t="n">
-        <v>2.193932810604526</v>
+        <v>2.959400431417178</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>growth_rate_factor</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>start_year</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>start_multiplier</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>multiplier_2050</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>annualised_growth_rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1.471446502093358</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.752303348613496</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.006741281978959623</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.471446502093358</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2.086767695049543</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.01352800884063932</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.471446502093358</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2.485071672406462</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.0203604869418077</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Very High</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.471446502093358</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2.959400431417178</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.02723902470447093</v>
       </c>
     </row>
   </sheetData>

</xml_diff>